<commit_message>
Verification layer: citation check, source register, status panel, push gate
- citation_check.py grades every evidence quote against its cited page
  (KB, original PDF or spreadsheet); visual sign-offs for chart images and
  font-encoded filings. Both reports pass.
- source_register.py hashes every input and confirms each knowledge base
  was built from it.
- validate_report.py: one status per report (PASS WITH NOTES for both),
  published on the live page and in each audit folder.
- hooks/pre-push blocks a push unless the self-test and every report
  validation pass.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/ADANIPORTS/Adani_Ports_and_Special_Economic_Zone_Ltd_ERIP_Model.xlsx
+++ b/reports/ADANIPORTS/Adani_Ports_and_Special_Economic_Zone_Ltd_ERIP_Model.xlsx
@@ -1964,11 +1964,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="0"/>
-        <c:axId val="70133606"/>
-        <c:axId val="44563335"/>
+        <c:axId val="40744974"/>
+        <c:axId val="447348"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="70133606"/>
+        <c:axId val="40744974"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -2001,7 +2001,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="44563335"/>
+        <c:crossAx val="447348"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2009,7 +2009,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="44563335"/>
+        <c:axId val="447348"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2042,7 +2042,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="70133606"/>
+        <c:crossAx val="40744974"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>